<commit_message>
prediction data and retrain button is displayed
</commit_message>
<xml_diff>
--- a/database/sample.xlsx
+++ b/database/sample.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Projects\ahadu_pulse\database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AhaduBank\Projects\AI Project\DigitalAIProject-API\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9070"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -418,9 +418,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:X4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -491,7 +491,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -562,7 +562,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -633,12 +633,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
       <c r="B4" s="1">
-        <v>46086</v>
+        <v>46210</v>
       </c>
       <c r="C4">
         <v>654</v>

</xml_diff>